<commit_message>
Changes to the framework toolbox to include calculation rules in the specifications
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/sfdr/sfdr.xlsx
+++ b/dataland-framework-toolbox/inputs/sfdr/sfdr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d40006\Documents\Dataland Project\Dataland\dataland-framework-toolbox\inputs\sfdr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dataland\datalandAlternative\dataland-framework-toolbox\inputs\sfdr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A91B7D7-4F81-46BF-99BF-699B9FC8F694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF6A987-99F1-4D4E-9B94-CF9C4465A6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64EA21DF-A91B-4C8A-A36C-EACA4F178F40}"/>
+    <workbookView xWindow="63890" yWindow="-10810" windowWidth="38620" windowHeight="21100" xr2:uid="{64EA21DF-A91B-4C8A-A36C-EACA4F178F40}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="2" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="438">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -1377,6 +1377,12 @@
   </si>
   <si>
     <t>Scope 2 greenhouse gas emissions in tonnes from the consumption of purchased electricity, steam, or other sources of energy computed using the market-based method (equity share approach preferably used).</t>
+  </si>
+  <si>
+    <t>Field Calculation</t>
+  </si>
+  <si>
+    <t>Sum: [extendedDecimalScope1GhgEmissionsInTonnes;extendedDecimalScope2GhgEmissionsInTonnes]; Division: [example1,example2]</t>
   </si>
 </sst>
 </file>
@@ -1794,17 +1800,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBCA27A-793A-4293-9394-36A2BE726731}">
-  <dimension ref="A1:N114"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:O114"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="58.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1847,8 +1861,11 @@
       <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1886,7 +1903,7 @@
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:15">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1924,7 +1941,7 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:15">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1962,7 +1979,7 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:15">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1998,7 +2015,7 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
     </row>
-    <row r="6" spans="1:14" s="6" customFormat="1">
+    <row r="6" spans="1:15" s="6" customFormat="1">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -2033,7 +2050,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:14" s="6" customFormat="1">
+    <row r="7" spans="1:15" s="6" customFormat="1">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -2064,7 +2081,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:14" s="6" customFormat="1">
+    <row r="8" spans="1:15" s="6" customFormat="1">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -2108,7 +2125,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="9" spans="1:14" s="6" customFormat="1">
+    <row r="9" spans="1:15" s="6" customFormat="1">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -2152,7 +2169,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="10" spans="1:14" s="6" customFormat="1">
+    <row r="10" spans="1:15" s="6" customFormat="1">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -2184,8 +2201,11 @@
       <c r="K10" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" s="6" customFormat="1">
+      <c r="O10" s="6" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" s="6" customFormat="1">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -2218,7 +2238,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="6" customFormat="1">
+    <row r="12" spans="1:15" s="6" customFormat="1">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -2251,7 +2271,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:14" s="6" customFormat="1">
+    <row r="13" spans="1:15" s="6" customFormat="1">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -2286,7 +2306,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:14" s="6" customFormat="1">
+    <row r="14" spans="1:15" s="6" customFormat="1">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -2317,7 +2337,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:14" s="6" customFormat="1">
+    <row r="15" spans="1:15" s="6" customFormat="1">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -2348,7 +2368,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:14" s="6" customFormat="1">
+    <row r="16" spans="1:15" s="6" customFormat="1">
       <c r="A16" s="4">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Update eu-non-financial taxonomy tootltips and spelling error in "GHG intensity - scope 4"
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/sfdr/sfdr.xlsx
+++ b/dataland-framework-toolbox/inputs/sfdr/sfdr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\srv\data\dataland\dataland-framework-toolbox\inputs\sfdr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC97FBC-0DD9-4118-B187-D8039C864A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815CF9E9-3A7D-494B-AD1A-2F6BDD17ABFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Framework Data Model" sheetId="1" r:id="rId1"/>
@@ -316,9 +316,6 @@
     <t>GHG_INTENSITY_SCOPE_4_IN_T_PER_MIO_EUR_REVENUE</t>
   </si>
   <si>
-    <t>Tonnes of scope 4 GHG emissions per million EUR revenue. As per the GHG Protocol, Scope 4 refers to emissions avoided when a product is used as a substitute for other goods or services, providing the same functions with a lower carbon footprint.</t>
-  </si>
-  <si>
     <t>Fossil Fuel Sector Exposure</t>
   </si>
   <si>
@@ -1603,12 +1600,15 @@
       <t>Water Consumption</t>
     </r>
   </si>
+  <si>
+    <t>Tons of scope 4 GHG emissions per million EUR revenue. As per the GHG Protocol, Scope 4 refers to emissions avoided when a product is used as a substitute for other goods or services, providing the same functions with a lower carbon footprint.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2053,24 +2053,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P114"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="58.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="255.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="38.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="255.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2117,10 +2117,10 @@
         <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -2158,7 +2158,7 @@
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -2194,7 +2194,7 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -2230,7 +2230,7 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -2264,7 +2264,7 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
     </row>
-    <row r="6" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" s="6" customFormat="1">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>37</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4" t="s">
@@ -2297,7 +2297,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" s="6" customFormat="1">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>43</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4" t="s">
@@ -2328,7 +2328,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" s="6" customFormat="1">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>45</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4" t="s">
@@ -2361,7 +2361,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" s="6" customFormat="1">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>47</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4" t="s">
@@ -2394,7 +2394,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" s="6" customFormat="1">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>49</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4" t="s">
@@ -2425,7 +2425,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" s="6" customFormat="1">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4" t="s">
@@ -2456,7 +2456,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" s="6" customFormat="1">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -2473,7 +2473,7 @@
         <v>53</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4" t="s">
@@ -2487,7 +2487,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" s="6" customFormat="1">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>55</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4" t="s">
@@ -2520,7 +2520,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" s="6" customFormat="1">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>57</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4" t="s">
@@ -2551,7 +2551,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" s="6" customFormat="1">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -2562,13 +2562,13 @@
         <v>41</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4" t="s">
@@ -2582,7 +2582,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" s="6" customFormat="1">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>60</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4" t="s">
@@ -2613,7 +2613,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" s="6" customFormat="1">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>62</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4" t="s">
@@ -2644,7 +2644,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" s="6" customFormat="1">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>64</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4" t="s">
@@ -2675,7 +2675,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" s="6" customFormat="1">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" s="6" customFormat="1">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>69</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4" t="s">
@@ -2737,7 +2737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" s="6" customFormat="1">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -2754,7 +2754,7 @@
         <v>72</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4" t="s">
@@ -2768,7 +2768,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" s="6" customFormat="1">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>74</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4" t="s">
@@ -2799,7 +2799,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" s="6" customFormat="1">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>77</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4" t="s">
@@ -2830,7 +2830,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" s="6" customFormat="1">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>80</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4" t="s">
@@ -2861,7 +2861,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" s="6" customFormat="1">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>82</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4" t="s">
@@ -2892,7 +2892,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" s="6" customFormat="1">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>84</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
@@ -2923,7 +2923,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" s="6" customFormat="1">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2940,7 +2940,7 @@
         <v>86</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>87</v>
+        <v>391</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
@@ -2954,7 +2954,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" s="6" customFormat="1">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -2965,17 +2965,17 @@
         <v>41</v>
       </c>
       <c r="D28" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>89</v>
-      </c>
       <c r="F28" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G28"/>
       <c r="H28" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>19</v>
@@ -2985,7 +2985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" s="6" customFormat="1">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -2996,13 +2996,13 @@
         <v>41</v>
       </c>
       <c r="D29" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="F29" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="5" t="s">
@@ -3010,13 +3010,13 @@
       </c>
       <c r="I29" s="4"/>
       <c r="J29" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K29" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" s="6" customFormat="1">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -3027,13 +3027,13 @@
         <v>41</v>
       </c>
       <c r="D30" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="F30" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="5" t="s">
@@ -3041,13 +3041,13 @@
       </c>
       <c r="I30" s="4"/>
       <c r="J30" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" s="6" customFormat="1">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -3055,16 +3055,16 @@
         <v>34</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="E31" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="F31" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
@@ -3074,13 +3074,13 @@
         <v>39</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K31" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" s="6" customFormat="1">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -3088,16 +3088,16 @@
         <v>34</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D32" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>101</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
@@ -3107,13 +3107,13 @@
         <v>39</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K32" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" s="6" customFormat="1">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -3121,16 +3121,16 @@
         <v>34</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D33" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="F33" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3140,13 +3140,13 @@
         <v>39</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K33" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" s="6" customFormat="1">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -3154,16 +3154,16 @@
         <v>34</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D34" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="F34" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3173,30 +3173,30 @@
         <v>39</v>
       </c>
       <c r="J34" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" s="6" customFormat="1">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D35" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="K34" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="4">
-        <v>34</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D35" s="8" t="s">
+      <c r="E35" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="F35" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3206,13 +3206,13 @@
         <v>39</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K35" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" s="6" customFormat="1">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -3220,16 +3220,16 @@
         <v>34</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D36" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E36" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="F36" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3239,13 +3239,13 @@
         <v>39</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" s="6" customFormat="1">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -3253,20 +3253,20 @@
         <v>34</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D37" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="F37" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G37"/>
       <c r="H37" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>19</v>
@@ -3278,7 +3278,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" s="6" customFormat="1">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -3286,16 +3286,16 @@
         <v>34</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D38" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="F38" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
@@ -3305,13 +3305,13 @@
         <v>39</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K38" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" s="6" customFormat="1">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -3319,16 +3319,16 @@
         <v>34</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D39" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>117</v>
-      </c>
       <c r="F39" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
@@ -3338,13 +3338,13 @@
         <v>39</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K39" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" s="6" customFormat="1">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -3352,16 +3352,16 @@
         <v>34</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D40" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="F40" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
@@ -3371,13 +3371,13 @@
         <v>39</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" s="6" customFormat="1">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -3385,16 +3385,16 @@
         <v>34</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D41" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E41" s="1" t="s">
-        <v>121</v>
-      </c>
       <c r="F41" s="1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
@@ -3404,13 +3404,13 @@
         <v>39</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K41" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" s="6" customFormat="1">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -3418,16 +3418,16 @@
         <v>34</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D42" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E42" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="F42" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
@@ -3437,13 +3437,13 @@
         <v>39</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K42" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" s="6" customFormat="1">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -3451,16 +3451,16 @@
         <v>34</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D43" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="F43" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4" t="s">
@@ -3470,13 +3470,13 @@
         <v>39</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K43" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" s="6" customFormat="1">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -3484,16 +3484,16 @@
         <v>34</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D44" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="F44" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4" t="s">
@@ -3503,13 +3503,13 @@
         <v>39</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K44" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" s="6" customFormat="1">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -3517,16 +3517,16 @@
         <v>34</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D45" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E45" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="F45" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="4" t="s">
@@ -3536,13 +3536,13 @@
         <v>39</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K45" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" s="6" customFormat="1">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -3550,20 +3550,20 @@
         <v>34</v>
       </c>
       <c r="C46" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="E46" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E46" s="1" t="s">
-        <v>132</v>
-      </c>
       <c r="F46" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G46"/>
       <c r="H46" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I46" s="4" t="s">
         <v>19</v>
@@ -3575,7 +3575,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" s="6" customFormat="1">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -3583,20 +3583,20 @@
         <v>34</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D47" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E47" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="F47" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G47"/>
       <c r="H47" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>19</v>
@@ -3608,7 +3608,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" s="6" customFormat="1">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -3616,20 +3616,20 @@
         <v>34</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D48" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="F48" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G48" s="4"/>
       <c r="H48" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>19</v>
@@ -3641,7 +3641,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" s="6" customFormat="1">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -3649,20 +3649,20 @@
         <v>34</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D49" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="1" t="s">
-        <v>138</v>
-      </c>
       <c r="F49" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G49"/>
       <c r="H49" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>19</v>
@@ -3674,7 +3674,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" s="6" customFormat="1">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -3682,20 +3682,20 @@
         <v>34</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D50" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="1" t="s">
-        <v>140</v>
-      </c>
       <c r="F50" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G50"/>
       <c r="H50" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>19</v>
@@ -3707,7 +3707,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" s="6" customFormat="1">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -3715,20 +3715,20 @@
         <v>34</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D51" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E51" s="1" t="s">
-        <v>142</v>
-      </c>
       <c r="F51" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G51"/>
       <c r="H51" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>19</v>
@@ -3740,7 +3740,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" s="6" customFormat="1">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -3748,20 +3748,20 @@
         <v>34</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D52" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E52" s="1" t="s">
-        <v>144</v>
-      </c>
       <c r="F52" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G52"/>
       <c r="H52" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>19</v>
@@ -3773,7 +3773,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" s="6" customFormat="1">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -3781,20 +3781,20 @@
         <v>34</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D53" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E53" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E53" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="F53" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G53"/>
       <c r="H53" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>19</v>
@@ -3806,7 +3806,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" s="6" customFormat="1">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -3814,20 +3814,20 @@
         <v>34</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D54" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="F54" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G54"/>
       <c r="H54" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>19</v>
@@ -3839,7 +3839,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" s="6" customFormat="1">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -3847,20 +3847,20 @@
         <v>34</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D55" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E55" s="1" t="s">
-        <v>150</v>
-      </c>
       <c r="F55" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G55"/>
       <c r="H55" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>19</v>
@@ -3872,7 +3872,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" s="6" customFormat="1">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -3880,20 +3880,20 @@
         <v>34</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D56" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="E56" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E56" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="F56" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G56"/>
       <c r="H56" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>19</v>
@@ -3905,7 +3905,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" s="6" customFormat="1">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -3913,16 +3913,16 @@
         <v>34</v>
       </c>
       <c r="C57" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D57" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="D57" s="8" t="s">
+      <c r="E57" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="E57" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="F57" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57" s="4" t="s">
@@ -3938,7 +3938,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" s="6" customFormat="1">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -3946,16 +3946,16 @@
         <v>34</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="4" t="s">
@@ -3965,13 +3965,13 @@
         <v>39</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K58" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" s="6" customFormat="1">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -3979,16 +3979,16 @@
         <v>34</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D59" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E59" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="F59" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="4" t="s">
@@ -3998,13 +3998,13 @@
         <v>39</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K59" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" s="6" customFormat="1">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -4012,16 +4012,16 @@
         <v>34</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D60" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="E60" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="F60" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4" t="s">
@@ -4031,13 +4031,13 @@
         <v>39</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K60" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="61" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" s="6" customFormat="1">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -4045,20 +4045,20 @@
         <v>34</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D61" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E61" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="F61" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G61"/>
       <c r="H61" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>19</v>
@@ -4070,7 +4070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" s="6" customFormat="1">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -4078,20 +4078,20 @@
         <v>34</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D62" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E62" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="F62" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G62"/>
       <c r="H62" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>19</v>
@@ -4103,7 +4103,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" s="6" customFormat="1">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -4111,16 +4111,16 @@
         <v>34</v>
       </c>
       <c r="C63" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D63" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="D63" s="8" t="s">
+      <c r="E63" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E63" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="F63" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="4" t="s">
@@ -4136,7 +4136,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" s="6" customFormat="1">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -4144,16 +4144,16 @@
         <v>34</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D64" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E64" s="1" t="s">
-        <v>171</v>
-      </c>
       <c r="F64" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G64" s="4"/>
       <c r="H64" s="4" t="s">
@@ -4169,7 +4169,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" s="6" customFormat="1">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -4177,16 +4177,16 @@
         <v>34</v>
       </c>
       <c r="C65" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D65" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="D65" s="8" t="s">
+      <c r="E65" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="F65" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G65" s="4"/>
       <c r="H65" s="4" t="s">
@@ -4202,7 +4202,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" s="6" customFormat="1">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -4210,16 +4210,16 @@
         <v>34</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D66" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E66" s="1" t="s">
-        <v>176</v>
-      </c>
       <c r="F66" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G66" s="4"/>
       <c r="H66" s="4" t="s">
@@ -4235,7 +4235,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" s="6" customFormat="1">
       <c r="A67" s="4">
         <v>66</v>
       </c>
@@ -4243,16 +4243,16 @@
         <v>34</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D67" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="E67" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="E67" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="F67" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="G67" s="4"/>
       <c r="H67" s="4" t="s">
@@ -4268,7 +4268,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" s="6" customFormat="1">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -4276,20 +4276,20 @@
         <v>34</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D68" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="E68" s="1" t="s">
-        <v>180</v>
-      </c>
       <c r="F68" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G68"/>
       <c r="H68" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>19</v>
@@ -4301,28 +4301,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" s="6" customFormat="1">
       <c r="A69" s="4">
         <v>68</v>
       </c>
       <c r="B69" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C69" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C69" s="4" t="s">
+      <c r="D69" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="D69" s="8" t="s">
+      <c r="E69" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="E69" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="F69" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G69"/>
       <c r="H69" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>19</v>
@@ -4334,28 +4334,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" s="6" customFormat="1">
       <c r="A70" s="4">
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C70" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C70" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D70" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="E70" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E70" s="1" t="s">
-        <v>186</v>
-      </c>
       <c r="F70" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G70"/>
       <c r="H70" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>19</v>
@@ -4367,28 +4367,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" s="6" customFormat="1">
       <c r="A71" s="4">
         <v>70</v>
       </c>
       <c r="B71" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C71" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C71" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D71" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="E71" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E71" s="1" t="s">
+      <c r="F71" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="G71"/>
       <c r="H71" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>19</v>
@@ -4400,28 +4400,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" s="6" customFormat="1">
       <c r="A72" s="4">
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C72" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C72" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D72" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="E72" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E72" s="1" t="s">
-        <v>191</v>
-      </c>
       <c r="F72" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G72"/>
       <c r="H72" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>19</v>
@@ -4433,28 +4433,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" s="6" customFormat="1">
       <c r="A73" s="4">
         <v>72</v>
       </c>
       <c r="B73" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C73" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C73" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D73" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="E73" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="F73" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>194</v>
       </c>
       <c r="G73" s="5"/>
       <c r="H73" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>19</v>
@@ -4466,28 +4466,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" s="6" customFormat="1">
       <c r="A74" s="4">
         <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C74" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C74" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D74" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E74" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="E74" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="F74" s="1" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G74" s="5"/>
       <c r="H74" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>19</v>
@@ -4499,28 +4499,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" s="6" customFormat="1">
       <c r="A75" s="4">
         <v>74</v>
       </c>
       <c r="B75" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C75" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C75" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D75" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="E75" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="E75" s="1" t="s">
-        <v>198</v>
-      </c>
       <c r="F75" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G75" s="5"/>
       <c r="H75" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>19</v>
@@ -4532,28 +4532,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" s="6" customFormat="1">
       <c r="A76" s="4">
         <v>75</v>
       </c>
       <c r="B76" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C76" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C76" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D76" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="E76" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E76" s="1" t="s">
-        <v>200</v>
-      </c>
       <c r="F76" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="G76" s="4"/>
       <c r="H76" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>19</v>
@@ -4565,28 +4565,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" s="6" customFormat="1">
       <c r="A77" s="4">
         <v>76</v>
       </c>
       <c r="B77" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C77" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C77" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D77" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="E77" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="F77" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="G77" s="4"/>
       <c r="H77" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>19</v>
@@ -4598,28 +4598,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" s="6" customFormat="1">
       <c r="A78" s="4">
         <v>77</v>
       </c>
       <c r="B78" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C78" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C78" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D78" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="E78" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="E78" s="1" t="s">
-        <v>205</v>
-      </c>
       <c r="F78" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="G78"/>
       <c r="H78" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I78" s="4" t="s">
         <v>19</v>
@@ -4631,28 +4631,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" s="6" customFormat="1">
       <c r="A79" s="4">
         <v>78</v>
       </c>
       <c r="B79" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C79" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C79" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D79" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E79" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E79" s="1" t="s">
-        <v>207</v>
-      </c>
       <c r="F79" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G79"/>
       <c r="H79" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>19</v>
@@ -4664,28 +4664,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" s="6" customFormat="1">
       <c r="A80" s="4">
         <v>79</v>
       </c>
       <c r="B80" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C80" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C80" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D80" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="F80" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="G80" s="4"/>
       <c r="H80" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>19</v>
@@ -4697,28 +4697,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" s="6" customFormat="1">
       <c r="A81" s="4">
         <v>80</v>
       </c>
       <c r="B81" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C81" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C81" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D81" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="E81" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="E81" s="1" t="s">
+      <c r="F81" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="G81" s="4"/>
       <c r="H81" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>19</v>
@@ -4730,28 +4730,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" s="6" customFormat="1">
       <c r="A82" s="4">
         <v>81</v>
       </c>
       <c r="B82" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C82" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C82" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D82" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="F82" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="G82" s="4"/>
       <c r="H82" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>19</v>
@@ -4763,28 +4763,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" s="6" customFormat="1">
       <c r="A83" s="4">
         <v>82</v>
       </c>
       <c r="B83" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C83" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C83" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D83" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="E83" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="E83" s="1" t="s">
-        <v>218</v>
-      </c>
       <c r="F83" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="G83" s="5"/>
       <c r="H83" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>19</v>
@@ -4796,28 +4796,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" s="6" customFormat="1">
       <c r="A84" s="4">
         <v>83</v>
       </c>
       <c r="B84" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C84" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C84" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D84" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="E84" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="E84" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="F84" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G84"/>
       <c r="H84" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>19</v>
@@ -4829,28 +4829,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" s="6" customFormat="1">
       <c r="A85" s="4">
         <v>84</v>
       </c>
       <c r="B85" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C85" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C85" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D85" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E85" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="E85" s="1" t="s">
-        <v>222</v>
-      </c>
       <c r="F85" s="1" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G85"/>
       <c r="H85" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>19</v>
@@ -4862,28 +4862,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" s="6" customFormat="1">
       <c r="A86" s="4">
         <v>85</v>
       </c>
       <c r="B86" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C86" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C86" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D86" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="E86" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="E86" s="1" t="s">
-        <v>224</v>
-      </c>
       <c r="F86" s="1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G86" s="4"/>
       <c r="H86" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>39</v>
@@ -4895,28 +4895,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" s="6" customFormat="1">
       <c r="A87" s="4">
         <v>86</v>
       </c>
       <c r="B87" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C87" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C87" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D87" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="E87" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="E87" s="1" t="s">
-        <v>227</v>
-      </c>
       <c r="F87" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G87" s="4"/>
       <c r="H87" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>39</v>
@@ -4928,24 +4928,24 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" s="6" customFormat="1">
       <c r="A88" s="4">
         <v>87</v>
       </c>
       <c r="B88" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C88" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C88" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D88" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="E88" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E88" s="1" t="s">
-        <v>229</v>
-      </c>
       <c r="F88" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G88" s="4"/>
       <c r="H88" s="4" t="s">
@@ -4953,34 +4953,34 @@
       </c>
       <c r="I88" s="4"/>
       <c r="J88" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K88" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" s="6" customFormat="1">
       <c r="A89" s="4">
         <v>88</v>
       </c>
       <c r="B89" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C89" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C89" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D89" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="E89" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="E89" s="1" t="s">
-        <v>231</v>
-      </c>
       <c r="F89" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G89" s="4"/>
       <c r="H89" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>39</v>
@@ -4990,28 +4990,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" s="6" customFormat="1">
       <c r="A90" s="4">
         <v>89</v>
       </c>
       <c r="B90" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C90" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C90" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D90" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="E90" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E90" s="1" t="s">
-        <v>234</v>
-      </c>
       <c r="F90" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G90" s="4"/>
       <c r="H90" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I90" s="4" t="s">
         <v>39</v>
@@ -5021,28 +5021,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" s="6" customFormat="1">
       <c r="A91" s="4">
         <v>90</v>
       </c>
       <c r="B91" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C91" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C91" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D91" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="E91" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="E91" s="1" t="s">
-        <v>236</v>
-      </c>
       <c r="F91" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G91" s="4"/>
       <c r="H91" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I91" s="4" t="s">
         <v>39</v>
@@ -5052,28 +5052,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" s="6" customFormat="1">
       <c r="A92" s="4">
         <v>91</v>
       </c>
       <c r="B92" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C92" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C92" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D92" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="E92" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E92" s="1" t="s">
-        <v>238</v>
-      </c>
       <c r="F92" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G92" s="4"/>
       <c r="H92" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I92" s="4" t="s">
         <v>39</v>
@@ -5083,94 +5083,94 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" s="6" customFormat="1">
       <c r="A93" s="4">
         <v>92</v>
       </c>
       <c r="B93" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C93" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C93" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D93" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="E93" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="E93" s="1" t="s">
-        <v>240</v>
-      </c>
       <c r="F93" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G93" s="4"/>
       <c r="H93" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K93" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" s="6" customFormat="1">
       <c r="A94" s="4">
         <v>93</v>
       </c>
       <c r="B94" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C94" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C94" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D94" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="E94" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E94" s="1" t="s">
-        <v>243</v>
-      </c>
       <c r="F94" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G94" s="4"/>
       <c r="H94" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J94" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K94" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" s="6" customFormat="1">
       <c r="A95" s="4">
         <v>94</v>
       </c>
       <c r="B95" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C95" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C95" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D95" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="E95" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="E95" s="1" t="s">
-        <v>245</v>
-      </c>
       <c r="F95" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G95"/>
       <c r="H95" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I95" s="4" t="s">
         <v>19</v>
@@ -5182,28 +5182,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" s="6" customFormat="1">
       <c r="A96" s="4">
         <v>95</v>
       </c>
       <c r="B96" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C96" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C96" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D96" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="E96" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="E96" s="1" t="s">
-        <v>247</v>
-      </c>
       <c r="F96" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G96"/>
       <c r="H96" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>19</v>
@@ -5215,24 +5215,24 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" s="6" customFormat="1">
       <c r="A97" s="4">
         <v>96</v>
       </c>
       <c r="B97" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C97" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C97" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D97" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="E97" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="E97" s="1" t="s">
-        <v>249</v>
-      </c>
       <c r="F97" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G97" s="4"/>
       <c r="H97" s="4" t="s">
@@ -5246,24 +5246,24 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" s="6" customFormat="1">
       <c r="A98" s="4">
         <v>97</v>
       </c>
       <c r="B98" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C98" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C98" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D98" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="E98" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="E98" s="1" t="s">
-        <v>251</v>
-      </c>
       <c r="F98" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G98" s="4"/>
       <c r="H98" s="4" t="s">
@@ -5273,34 +5273,34 @@
         <v>39</v>
       </c>
       <c r="J98" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="K98" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" s="6" customFormat="1">
       <c r="A99" s="4">
         <v>98</v>
       </c>
       <c r="B99" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C99" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C99" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D99" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="E99" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="E99" s="1" t="s">
-        <v>254</v>
-      </c>
       <c r="F99" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G99"/>
       <c r="H99" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I99" s="4" t="s">
         <v>19</v>
@@ -5312,28 +5312,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" s="6" customFormat="1">
       <c r="A100" s="4">
         <v>99</v>
       </c>
       <c r="B100" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C100" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C100" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D100" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="E100" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="E100" s="1" t="s">
-        <v>256</v>
-      </c>
       <c r="F100" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G100"/>
       <c r="H100" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I100" s="4" t="s">
         <v>19</v>
@@ -5345,28 +5345,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" s="6" customFormat="1">
       <c r="A101" s="4">
         <v>100</v>
       </c>
       <c r="B101" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C101" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C101" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D101" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="E101" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="E101" s="1" t="s">
-        <v>258</v>
-      </c>
       <c r="F101" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G101"/>
       <c r="H101" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I101" s="4" t="s">
         <v>19</v>
@@ -5378,28 +5378,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" s="6" customFormat="1">
       <c r="A102" s="4">
         <v>101</v>
       </c>
       <c r="B102" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C102" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C102" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D102" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="E102" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="E102" s="1" t="s">
-        <v>260</v>
-      </c>
       <c r="F102" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G102" s="4"/>
       <c r="H102" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I102" s="4" t="s">
         <v>39</v>
@@ -5411,28 +5411,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" s="6" customFormat="1">
       <c r="A103" s="4">
         <v>102</v>
       </c>
       <c r="B103" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C103" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C103" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D103" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="E103" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="E103" s="1" t="s">
-        <v>262</v>
-      </c>
       <c r="F103" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G103" s="4"/>
       <c r="H103" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I103" s="4" t="s">
         <v>39</v>
@@ -5444,24 +5444,24 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:11" s="6" customFormat="1">
       <c r="A104" s="4">
         <v>103</v>
       </c>
       <c r="B104" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C104" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C104" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="D104" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="E104" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="E104" s="1" t="s">
-        <v>264</v>
-      </c>
       <c r="F104" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G104" s="4"/>
       <c r="H104" s="4" t="s">
@@ -5475,28 +5475,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:11" s="6" customFormat="1">
       <c r="A105" s="4">
         <v>104</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C105" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D105" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="D105" s="8" t="s">
+      <c r="E105" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="E105" s="1" t="s">
+      <c r="F105" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="F105" s="1" t="s">
-        <v>268</v>
       </c>
       <c r="G105" s="5"/>
       <c r="H105" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I105" s="4" t="s">
         <v>19</v>
@@ -5508,28 +5508,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:11" s="6" customFormat="1">
       <c r="A106" s="4">
         <v>105</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C106" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="D106" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="D106" s="8" t="s">
+      <c r="E106" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="E106" s="1" t="s">
-        <v>271</v>
-      </c>
       <c r="F106" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G106"/>
       <c r="H106" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I106" s="4" t="s">
         <v>19</v>
@@ -5541,28 +5541,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:11" s="6" customFormat="1">
       <c r="A107" s="4">
         <v>106</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D107" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="E107" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="E107" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="F107" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G107"/>
       <c r="H107" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I107" s="4" t="s">
         <v>19</v>
@@ -5574,28 +5574,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:11" s="6" customFormat="1">
       <c r="A108" s="4">
         <v>107</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D108" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="E108" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="E108" s="1" t="s">
-        <v>275</v>
-      </c>
       <c r="F108" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G108"/>
       <c r="H108" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I108" s="4" t="s">
         <v>19</v>
@@ -5607,28 +5607,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:11" s="6" customFormat="1">
       <c r="A109" s="4">
         <v>108</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D109" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="E109" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="E109" s="1" t="s">
-        <v>277</v>
-      </c>
       <c r="F109" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="G109"/>
       <c r="H109" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I109" s="4" t="s">
         <v>19</v>
@@ -5640,28 +5640,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:11" s="6" customFormat="1">
       <c r="A110" s="4">
         <v>109</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D110" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="E110" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="E110" s="1" t="s">
-        <v>279</v>
-      </c>
       <c r="F110" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G110"/>
       <c r="H110" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I110" s="4" t="s">
         <v>19</v>
@@ -5673,28 +5673,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:11" s="6" customFormat="1">
       <c r="A111" s="4">
         <v>110</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D111" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="E111" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="E111" s="1" t="s">
-        <v>281</v>
-      </c>
       <c r="F111" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="G111" s="4"/>
       <c r="H111" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I111" s="4" t="s">
         <v>39</v>
@@ -5706,28 +5706,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="112" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:11" s="6" customFormat="1">
       <c r="A112" s="4">
         <v>111</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C112" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D112" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="D112" s="8" t="s">
+      <c r="E112" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="E112" s="1" t="s">
-        <v>284</v>
-      </c>
       <c r="F112" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G112" s="4"/>
       <c r="H112" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>39</v>
@@ -5739,28 +5739,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:11" s="6" customFormat="1">
       <c r="A113" s="4">
         <v>112</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D113" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="E113" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="E113" s="1" t="s">
-        <v>286</v>
-      </c>
       <c r="F113" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G113" s="4"/>
       <c r="H113" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I113" s="4" t="s">
         <v>39</v>
@@ -5772,28 +5772,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="114" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:11" s="6" customFormat="1">
       <c r="A114" s="4">
         <v>113</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D114" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="E114" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="E114" s="1" t="s">
-        <v>288</v>
-      </c>
       <c r="F114" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G114" s="4"/>
       <c r="H114" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I114" s="4" t="s">
         <v>39</v>

</xml_diff>